<commit_message>
Migrate Komnata runtime from SQLite to Neon and fix PostgreSQL queries
</commit_message>
<xml_diff>
--- a/komnata_backup.xlsx
+++ b/komnata_backup.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -475,11 +475,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>prod</t>
+          <t>sql</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -498,29 +498,25 @@
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-05-01 10:17:26</t>
+          <t>2026-05-04 13:39:11</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-05-01 10:17:26</t>
+          <t>2026-05-04 13:39:11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>produkt</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
+          <t>prod</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
@@ -536,18 +532,18 @@
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-05-01 10:02:28</t>
+          <t>2026-05-01 10:17:26</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-05-01 10:13:56</t>
+          <t>2026-05-01 10:17:26</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -556,45 +552,45 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Regał 3</t>
+          <t>Regał 1</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0B</t>
+          <t>0A</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-05-01 09:30:42</t>
+          <t>2026-05-01 10:02:28</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-05-01 10:01:18</t>
+          <t>2026-05-01 10:13:56</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>produkt 1.05</t>
+          <t>produkt</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -606,31 +602,35 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0A</t>
+          <t>0B</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-05-01 09:25:48</t>
+          <t>2026-05-01 09:30:42</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-05-01 09:59:34</t>
+          <t>2026-05-01 10:01:18</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PRODUKT 30.04</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>produkt 1.05</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
@@ -640,28 +640,28 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0B</t>
+          <t>0A</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-04-30 14:55:06</t>
+          <t>2026-05-01 09:25:48</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-04-30 14:55:06</t>
+          <t>2026-05-01 09:59:34</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>DODAJ TEST MODYFIKACJA</t>
+          <t>PRODUKT 30.04</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -674,28 +674,28 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>1A</t>
+          <t>0B</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-04-30 14:50:23</t>
+          <t>2026-04-30 14:55:06</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-04-30 14:50:23</t>
+          <t>2026-04-30 14:55:06</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>YEST 2</t>
+          <t>DODAJ TEST MODYFIKACJA</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -714,60 +714,56 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-04-30 14:41:45</t>
+          <t>2026-04-30 14:50:23</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-04-30 14:41:45</t>
+          <t>2026-04-30 14:50:23</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>TEST KOPII</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+          <t>YEST 2</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>regał 100</t>
+          <t>Regał 3</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0A</t>
+          <t>1A</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-04-29 14:56:37</t>
+          <t>2026-04-30 14:41:45</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-04-29 14:58:46</t>
+          <t>2026-04-30 14:41:45</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>FARBA</t>
+          <t>TEST KOPII</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -779,29 +775,29 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Regał 3</t>
+          <t>regał 100</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>1B</t>
+          <t>0A</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-04-29 14:22:35</t>
+          <t>2026-04-29 14:56:37</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-04-29 14:31:30</t>
+          <t>2026-04-29 14:58:46</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -822,36 +818,40 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>1A</t>
+          <t>1B</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-04-14 02:45:55</t>
+          <t>2026-04-29 14:22:35</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-04-29 14:31:10</t>
+          <t>2026-04-29 14:31:30</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>dRVA</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
+          <t>FARBA</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Regał 1</t>
+          <t>Regał 3</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -862,22 +862,22 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-04-14 02:41:43</t>
+          <t>2026-04-14 02:45:55</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-04-14 02:41:43</t>
+          <t>2026-04-29 14:31:10</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>niniin</t>
+          <t>dRVA</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -885,45 +885,37 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Regał 88</t>
+          <t>Regał 1</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>3A</t>
+          <t>1A</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-04-14 02:07:38</t>
+          <t>2026-04-14 02:41:43</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-04-14 02:07:38</t>
+          <t>2026-04-14 02:41:43</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>rag</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
+          <t>niniin</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
@@ -932,32 +924,40 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>0A</t>
+          <t>3A</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-04-14 01:50:45</t>
+          <t>2026-04-14 02:07:38</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-04-29 14:31:59</t>
+          <t>2026-04-14 02:07:38</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>test godziny</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
@@ -966,28 +966,28 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>1A</t>
+          <t>0A</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-04-14 01:47:23</t>
+          <t>2026-04-14 01:50:45</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-04-14 01:47:23</t>
+          <t>2026-04-29 14:31:59</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>farba tgest</t>
+          <t>test godziny</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -1000,16 +1000,50 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>0A</t>
+          <t>1A</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
+          <t>2026-04-14 01:47:23</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2026-04-14 01:47:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>3</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>farba tgest</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Regał 88</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>0A</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
           <t>2026-04-14 01:37:52</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>2026-04-14 01:37:52</t>
         </is>

</xml_diff>